<commit_message>
feat: add the projects info to the dialog
</commit_message>
<xml_diff>
--- a/arquivos_apoio/Gestão MEG.xlsx
+++ b/arquivos_apoio/Gestão MEG.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ml0559\Documents\Projetos\node\dash_melhorias\dash_melhorias\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ml0559\Documents\Projetos\node\dash_melhorias\dash_melhorias\arquivos_apoio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74A8211-5F11-41B5-A3FB-D88101F47C25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49A79C1D-2CCD-4A9D-8135-13BAD7DA5209}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plano" sheetId="1" state="hidden" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <sheet name="Planilha1" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dados Consolidados'!$A$1:$S$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dados Consolidados'!$A$1:$S$125</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Tarefas!$A$1:$T$124</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -2073,7 +2073,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:T125"/>
+  <dimension ref="A1:T124"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.875" customWidth="1"/>
@@ -9558,13 +9558,8 @@
         <v>7.44</v>
       </c>
     </row>
-    <row r="125" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="T125">
-        <v>565.41999999999996</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:S124" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A1:S125" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <headerFooter>

</xml_diff>